<commit_message>
feat: add Insurance Planning calculator to Planning page
- New '🔒 Insurance Planning' tab (4th tab)
- Calculates: Life/Death Benefit, CI, TPD, PA coverage needs
- Life need = income replacement + outstanding debts + final expenses
- CI = max(5x annual income, RM 200K)
- TPD = same as Life; PA = 2x annual income
- Coverage gap bar charts with % filled
- Overall protection score (0-100%)
- Premium budget check (10% of income rule)
- Recommended coverage summary table
- PDF export via existing downloadPDF helper
- Supports existing client (pre-fill from Notion) or fresh prospect

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/1_Clients_Database.xlsx
+++ b/notion-import-templates/1_Clients_Database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E31C45D-54D3-48BF-A699-7D0209D40864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 READ ME FIRST" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="81">
   <si>
     <t/>
   </si>
@@ -172,6 +172,9 @@
     <t>e.g. client@email.com</t>
   </si>
   <si>
+    <t>⬅ EXAMPLE — DELETE THIS ROW BEFORE IMPORTING</t>
+  </si>
+  <si>
     <t>Active</t>
   </si>
   <si>
@@ -181,6 +184,12 @@
     <t>Moderate</t>
   </si>
   <si>
+    <t>1984-06-15</t>
+  </si>
+  <si>
+    <t>2024-01-10</t>
+  </si>
+  <si>
     <t>2025-08-16</t>
   </si>
   <si>
@@ -190,6 +199,12 @@
     <t>Retirement,Property</t>
   </si>
   <si>
+    <t>+60123456789</t>
+  </si>
+  <si>
+    <t>ahmad@email.com</t>
+  </si>
+  <si>
     <t>LEONG CHEE KEONG</t>
   </si>
   <si>
@@ -235,17 +250,35 @@
     <t>60124939349</t>
   </si>
   <si>
-    <t>Retirement,Property,Education</t>
-  </si>
-  <si>
-    <t>Retirement</t>
+    <t>LOH SHI SHENG</t>
+  </si>
+  <si>
+    <t>lohshisheng@gmail.com</t>
+  </si>
+  <si>
+    <t>WONG CHENG YEAT</t>
+  </si>
+  <si>
+    <t>JACKWCY28@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>WONG CHENG LIANG</t>
+  </si>
+  <si>
+    <t>COOZAUTO@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>KOK HUEI MIN</t>
+  </si>
+  <si>
+    <t>HMKOK5637@GMAIL.COM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -258,73 +291,94 @@
       <sz val="16"/>
       <color rgb="FF0A4A14"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF4A7A4E"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0F2012"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1A1A1A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF2D6A35"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1565C0"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFC62828"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FFE8F5EA"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFA8D5AC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFE8F5EA"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF555555"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF1565C0"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF1565C0"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -432,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -467,7 +521,12 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -477,8 +536,11 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -820,14 +882,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -838,7 +900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -849,7 +911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -860,7 +922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -871,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -882,7 +944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -893,7 +955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -904,7 +966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -915,7 +977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -926,7 +988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -937,7 +999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -948,7 +1010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -959,7 +1021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -970,7 +1032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -981,7 +1043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -992,7 +1054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1003,7 +1065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1014,7 +1076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1025,7 +1087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1036,7 +1098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1047,7 +1109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1066,57 +1128,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M54"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:M55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="44" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="30" customWidth="1"/>
+    <col min="1" max="1" width="36" style="14" customWidth="1"/>
+    <col min="2" max="2" width="14" style="14" customWidth="1"/>
+    <col min="3" max="3" width="18" style="14" customWidth="1"/>
+    <col min="4" max="4" width="16" style="14" customWidth="1"/>
+    <col min="5" max="5" width="14" style="14" customWidth="1"/>
+    <col min="6" max="6" width="20" style="14" customWidth="1"/>
+    <col min="7" max="7" width="16" style="14" customWidth="1"/>
+    <col min="8" max="10" width="18" style="14" customWidth="1"/>
+    <col min="11" max="11" width="44" style="14" customWidth="1"/>
+    <col min="12" max="12" width="20" style="17" customWidth="1"/>
+    <col min="13" max="13" width="30" style="14" customWidth="1"/>
+    <col min="14" max="16384" width="8.7265625" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-    </row>
-    <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="15" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+    </row>
+    <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-    </row>
-    <row r="3" spans="1:13" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+    </row>
+    <row r="3" spans="1:13" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>24</v>
       </c>
@@ -1157,7 +1220,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>37</v>
       </c>
@@ -1198,257 +1261,284 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row r="5" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="13">
+        <v>250000</v>
+      </c>
+      <c r="F5" s="13">
+        <v>12000</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="K5" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="L5" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5">
-        <v>15000</v>
-      </c>
-      <c r="G5" s="12">
+      <c r="G6" s="18">
         <v>31769</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H6" s="18">
         <v>42115</v>
       </c>
-      <c r="I5" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K5" t="s">
-        <v>52</v>
-      </c>
-      <c r="L5" t="s">
+      <c r="L6" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="M6" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="18">
+        <v>28299</v>
+      </c>
+      <c r="H7" s="18">
+        <v>44249</v>
+      </c>
+      <c r="L7" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="M5" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B8" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6">
-        <v>30000</v>
-      </c>
-      <c r="G6" s="12">
-        <v>28299</v>
-      </c>
-      <c r="H6" s="12">
-        <v>44249</v>
-      </c>
-      <c r="I6" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="G8" s="18">
+        <v>30150</v>
+      </c>
+      <c r="H8" s="18">
+        <v>44252</v>
+      </c>
+      <c r="L8" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="M8" s="14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="18">
+        <v>28742</v>
+      </c>
+      <c r="H9" s="18">
+        <v>44490</v>
+      </c>
+      <c r="L9" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="M9" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="L6" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="M6" s="13" t="s">
+    </row>
+    <row r="10" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B10" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7">
-        <v>20000</v>
-      </c>
-      <c r="G7" s="12">
-        <v>30150</v>
-      </c>
-      <c r="H7" s="12">
-        <v>44252</v>
-      </c>
-      <c r="I7" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" t="s">
-        <v>68</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="M7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="G10" s="18">
+        <v>24020</v>
+      </c>
+      <c r="H10" s="18">
+        <v>42235</v>
+      </c>
+      <c r="L10" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8">
-        <v>15000</v>
-      </c>
-      <c r="G8" s="12">
-        <v>28742</v>
-      </c>
-      <c r="H8" s="12">
-        <v>44490</v>
-      </c>
-      <c r="I8" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="J8" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" t="s">
-        <v>69</v>
-      </c>
-      <c r="L8" t="s">
-        <v>64</v>
-      </c>
-      <c r="M8" s="13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="G11" s="18">
+        <v>31672</v>
+      </c>
+      <c r="H11" s="18">
+        <v>42996</v>
+      </c>
+      <c r="L11" s="17">
+        <v>60127264633</v>
+      </c>
+      <c r="M11" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9">
-        <v>5000</v>
-      </c>
-      <c r="G9" s="12">
-        <v>24020</v>
-      </c>
-      <c r="H9" s="12">
-        <v>42235</v>
-      </c>
-      <c r="I9" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K9" t="s">
-        <v>69</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="11" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="12" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="13" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="14" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="15" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="16" spans="1:13" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="17" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="18" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="19" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="20" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="21" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="22" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="23" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="24" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="25" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="26" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="27" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="28" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="29" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="30" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="31" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="32" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="33" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="34" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="35" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="36" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="37" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="38" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="39" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="40" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="41" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="42" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="43" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="44" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="45" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="46" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="47" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="48" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="49" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="50" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="51" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="52" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="53" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="54" ht="22.05" customHeight="1" x14ac:dyDescent="0.45"/>
+      <c r="G12" s="18">
+        <v>31359</v>
+      </c>
+      <c r="H12" s="18">
+        <v>41636</v>
+      </c>
+      <c r="L12" s="17">
+        <v>60126617880</v>
+      </c>
+      <c r="M12" s="14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" s="18">
+        <v>31463</v>
+      </c>
+      <c r="H13" s="18">
+        <v>40752</v>
+      </c>
+      <c r="L13" s="17">
+        <v>60172292882</v>
+      </c>
+      <c r="M13" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G14" s="18">
+        <v>30494</v>
+      </c>
+      <c r="H14" s="18">
+        <v>40145</v>
+      </c>
+      <c r="L14" s="17">
+        <v>60166945993</v>
+      </c>
+      <c r="M14" s="14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="18" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="19" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="20" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="21" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="22" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="23" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="25" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="26" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="27" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="28" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="31" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="32" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="33" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="35" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="36" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="37" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="38" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="39" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="40" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="41" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="42" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="43" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="44" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="45" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="46" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="47" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="48" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="50" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="52" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="53" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="54" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="55" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B5:B54" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B6:B55" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Active,Prospect,Inactive"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C5:C54" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C6:C55" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Affluent,Mass Affluent,HNW,UHNW"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D10:D54" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D6:D55" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>"Conservative,Moderate,Aggressive"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G5:H54 I10:J54" xr:uid="{00000000-0002-0000-0100-000006000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G6:J55" xr:uid="{00000000-0002-0000-0100-000006000000}">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: Email Hub — Gmail integration with AI drafting and outbound compose
- lib/gmail.ts: OAuth2 auth, email list/thread/send, ARIA labels
- lib/emailClassifier.ts: Gemini classify, summarise, draft reply, draft new
- lib/getAdvisorConfig.ts: add gmail fields + saveGmailToken/saveInstitutions
- API routes: /auth /callback /list /thread /send /draft /close /institutions
- EmailHubPage: split-pane inbox with status tabs, AI summary panel, reply flow
- ComposeEmailModal: outbound new email with institution picker + AI draft
- Sidebar: Email Hub nav item added
- package.json: googleapis dependency

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/1_Clients_Database.xlsx
+++ b/notion-import-templates/1_Clients_Database.xlsx
@@ -1,18 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30125"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D563757-2660-4B04-8139-2E36AF5670CE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 READ ME FIRST" sheetId="1" r:id="rId1"/>
     <sheet name="Clients Data Entry" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -29,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="92">
   <si>
     <t/>
   </si>
@@ -172,113 +175,146 @@
     <t>e.g. client@email.com</t>
   </si>
   <si>
-    <t>⬅ EXAMPLE — DELETE THIS ROW BEFORE IMPORTING</t>
+    <t>DAMIEN NG TZE HOONG</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
+    <t>60107607223</t>
+  </si>
+  <si>
+    <t>dnth86@gmail.com</t>
+  </si>
+  <si>
+    <t>LEONG CHEE KEONG</t>
+  </si>
+  <si>
+    <t>60124303938</t>
+  </si>
+  <si>
+    <t>dleongck@gmail.com</t>
+  </si>
+  <si>
+    <t>NG MEI CHING</t>
+  </si>
+  <si>
+    <t>60124939349</t>
+  </si>
+  <si>
+    <t>ngmching@yahoo.com</t>
+  </si>
+  <si>
+    <t>KAREN CHEW AI LENG</t>
+  </si>
+  <si>
+    <t>60123959997</t>
+  </si>
+  <si>
+    <t>karenchew0909@yahoo.com</t>
+  </si>
+  <si>
+    <t>KAM BENG SIM</t>
+  </si>
+  <si>
+    <t>60122716391</t>
+  </si>
+  <si>
+    <t>lamlets@gmail.com</t>
+  </si>
+  <si>
+    <t>LOH SHI SHENG</t>
+  </si>
+  <si>
+    <t>lohshisheng@gmail.com</t>
+  </si>
+  <si>
+    <t>WONG CHENG YEAT</t>
+  </si>
+  <si>
+    <t>JACKWCY28@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>WONG CHENG LIANG</t>
+  </si>
+  <si>
+    <t>COOZAUTO@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>KOK HUEI MIN</t>
+  </si>
+  <si>
+    <t>HMKOK5637@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>DORIS CHIEW JING TZE</t>
+  </si>
+  <si>
     <t>Affluent</t>
   </si>
   <si>
+    <t>ahtze85@hotmail.com</t>
+  </si>
+  <si>
+    <t>TAN PIEH FANG</t>
+  </si>
+  <si>
+    <t>alicetan1973@gmail.com</t>
+  </si>
+  <si>
+    <t>LIM WOOI KHANG</t>
+  </si>
+  <si>
     <t>Moderate</t>
   </si>
   <si>
-    <t>1984-06-15</t>
-  </si>
-  <si>
-    <t>2024-01-10</t>
-  </si>
-  <si>
-    <t>2025-08-16</t>
-  </si>
-  <si>
-    <t>2026-08-16</t>
-  </si>
-  <si>
-    <t>Retirement,Property</t>
-  </si>
-  <si>
-    <t>+60123456789</t>
-  </si>
-  <si>
-    <t>ahmad@email.com</t>
-  </si>
-  <si>
-    <t>LEONG CHEE KEONG</t>
-  </si>
-  <si>
-    <t>NG MEI CHING</t>
-  </si>
-  <si>
-    <t>DAMIEN NG TZE HOONG</t>
-  </si>
-  <si>
-    <t>KAREN CHEW AI LENG</t>
-  </si>
-  <si>
-    <t>KAM BENG SIM</t>
-  </si>
-  <si>
-    <t>ngmching@yahoo.com</t>
-  </si>
-  <si>
-    <t>60107607223</t>
-  </si>
-  <si>
-    <t>dnth86@gmail.com</t>
-  </si>
-  <si>
-    <t>60124303938</t>
-  </si>
-  <si>
-    <t>dleongck@gmail.com</t>
-  </si>
-  <si>
-    <t>karenchew0909@yahoo.com</t>
-  </si>
-  <si>
-    <t>60123959997</t>
-  </si>
-  <si>
-    <t>60122716391</t>
-  </si>
-  <si>
-    <t>lamlets@gmail.com</t>
-  </si>
-  <si>
-    <t>60124939349</t>
-  </si>
-  <si>
-    <t>LOH SHI SHENG</t>
-  </si>
-  <si>
-    <t>lohshisheng@gmail.com</t>
-  </si>
-  <si>
-    <t>WONG CHENG YEAT</t>
-  </si>
-  <si>
-    <t>JACKWCY28@GMAIL.COM</t>
-  </si>
-  <si>
-    <t>WONG CHENG LIANG</t>
-  </si>
-  <si>
-    <t>COOZAUTO@GMAIL.COM</t>
-  </si>
-  <si>
-    <t>KOK HUEI MIN</t>
-  </si>
-  <si>
-    <t>HMKOK5637@GMAIL.COM</t>
+    <t>wk1168@gmail.com</t>
+  </si>
+  <si>
+    <t>LIM SHENG YEE</t>
+  </si>
+  <si>
+    <t>jessicalim14@gmail.com</t>
+  </si>
+  <si>
+    <t>HOO PENG YAN</t>
+  </si>
+  <si>
+    <t>bryanhoo111@gmail.com</t>
+  </si>
+  <si>
+    <t>TOH SHU HUA</t>
+  </si>
+  <si>
+    <t>tohshuhua@gmail.com</t>
+  </si>
+  <si>
+    <t>TAN LI YING</t>
+  </si>
+  <si>
+    <t>jatmee_tan86@yahoo.com</t>
+  </si>
+  <si>
+    <t>CHAN CHEE KENG</t>
+  </si>
+  <si>
+    <t>ken_chan6861@yahoo.com</t>
+  </si>
+  <si>
+    <t>LIU KAI YOU</t>
+  </si>
+  <si>
+    <t>Aggressive</t>
+  </si>
+  <si>
+    <t>kayu1204@yahoo.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,19 +402,12 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FF1565C0"/>
-      <name val="Arial"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF1565C0"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="10">
@@ -429,7 +458,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -467,26 +496,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBAD7F5"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBAD7F5"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBAD7F5"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBAD7F5"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -521,13 +536,16 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -536,14 +554,9 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -882,14 +895,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15" customHeight="1">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -900,7 +913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="10.15" customHeight="1">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -911,7 +924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="11.1" customHeight="1">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -922,7 +935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="10.15" customHeight="1">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -933,7 +946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="10.15" customHeight="1">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -944,7 +957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="10.15" customHeight="1">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -955,7 +968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="10.15" customHeight="1">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -966,7 +979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="10.15" customHeight="1">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -977,7 +990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="10.15" customHeight="1">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -988,7 +1001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="10.15" customHeight="1">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -999,7 +1012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="11.1" customHeight="1">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1010,7 +1023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="10.15" customHeight="1">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1021,7 +1034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="10.15" customHeight="1">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1032,7 +1045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="10.15" customHeight="1">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1043,7 +1056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="10.15" customHeight="1">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1054,7 +1067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="10.15" customHeight="1">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1065,7 +1078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="11" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" ht="11.1" customHeight="1">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1076,7 +1089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" ht="10.15" customHeight="1">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1087,7 +1100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" ht="10.15" customHeight="1">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1098,7 +1111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" ht="10.15" customHeight="1">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1109,7 +1122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="10" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="10.15" customHeight="1">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1128,58 +1141,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M55"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:M54"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="36" style="14" customWidth="1"/>
-    <col min="2" max="2" width="14" style="14" customWidth="1"/>
-    <col min="3" max="3" width="18" style="14" customWidth="1"/>
-    <col min="4" max="4" width="16" style="14" customWidth="1"/>
-    <col min="5" max="5" width="14" style="14" customWidth="1"/>
-    <col min="6" max="6" width="20" style="14" customWidth="1"/>
-    <col min="7" max="7" width="16" style="14" customWidth="1"/>
-    <col min="8" max="10" width="18" style="14" customWidth="1"/>
-    <col min="11" max="11" width="44" style="14" customWidth="1"/>
-    <col min="12" max="12" width="20" style="17" customWidth="1"/>
-    <col min="13" max="13" width="30" style="14" customWidth="1"/>
-    <col min="14" max="16384" width="8.7265625" style="14"/>
+    <col min="1" max="1" width="36" style="12" customWidth="1"/>
+    <col min="2" max="2" width="14" style="12" customWidth="1"/>
+    <col min="3" max="3" width="18" style="12" customWidth="1"/>
+    <col min="4" max="4" width="16" style="12" customWidth="1"/>
+    <col min="5" max="5" width="14" style="12" customWidth="1"/>
+    <col min="6" max="6" width="20" style="12" customWidth="1"/>
+    <col min="7" max="7" width="16" style="12" customWidth="1"/>
+    <col min="8" max="10" width="18" style="12" customWidth="1"/>
+    <col min="11" max="11" width="44" style="12" customWidth="1"/>
+    <col min="12" max="12" width="20" style="13" customWidth="1"/>
+    <col min="13" max="13" width="30" style="12" customWidth="1"/>
+    <col min="14" max="16384" width="8.7109375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:13" ht="28.15" customHeight="1">
+      <c r="A1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-    </row>
-    <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+    </row>
+    <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1">
+      <c r="A2" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="16"/>
-    </row>
-    <row r="3" spans="1:13" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+    </row>
+    <row r="3" spans="1:13" ht="32.1" customHeight="1">
       <c r="A3" s="10" t="s">
         <v>24</v>
       </c>
@@ -1220,7 +1233,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="28.15" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>37</v>
       </c>
@@ -1261,287 +1274,476 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="22.15" customHeight="1">
       <c r="A5" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="G5" s="14">
+        <v>31769</v>
+      </c>
+      <c r="H5" s="14">
+        <v>42115</v>
+      </c>
+      <c r="L5" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="M5" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="13">
-        <v>250000</v>
-      </c>
-      <c r="F5" s="13">
-        <v>12000</v>
-      </c>
-      <c r="G5" s="13" t="s">
+    </row>
+    <row r="6" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A6" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="B6" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="14">
+        <v>28299</v>
+      </c>
+      <c r="H6" s="14">
+        <v>44249</v>
+      </c>
+      <c r="L6" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="M6" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="J5" s="13" t="s">
+    </row>
+    <row r="7" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A7" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="B7" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="14">
+        <v>30150</v>
+      </c>
+      <c r="H7" s="14">
+        <v>44252</v>
+      </c>
+      <c r="L7" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="M7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="M5" s="13" t="s">
+    </row>
+    <row r="8" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A8" s="12" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="B8" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="14">
+        <v>28742</v>
+      </c>
+      <c r="H8" s="14">
+        <v>44490</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A9" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="18">
-        <v>31769</v>
-      </c>
-      <c r="H6" s="18">
-        <v>42115</v>
-      </c>
-      <c r="L6" s="17" t="s">
+      <c r="G9" s="14">
+        <v>24020</v>
+      </c>
+      <c r="H9" s="14">
+        <v>42235</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A10" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="14">
+        <v>31672</v>
+      </c>
+      <c r="H10" s="14">
+        <v>42996</v>
+      </c>
+      <c r="L10" s="13">
+        <v>60127264633</v>
+      </c>
+      <c r="M10" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="M6" s="14" t="s">
+    </row>
+    <row r="11" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A11" s="12" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="18">
-        <v>28299</v>
-      </c>
-      <c r="H7" s="18">
-        <v>44249</v>
-      </c>
-      <c r="L7" s="17" t="s">
+      <c r="G11" s="14">
+        <v>31359</v>
+      </c>
+      <c r="H11" s="14">
+        <v>41636</v>
+      </c>
+      <c r="L11" s="13">
+        <v>60126617880</v>
+      </c>
+      <c r="M11" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="M7" s="14" t="s">
+    </row>
+    <row r="12" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A12" s="12" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="18">
-        <v>30150</v>
-      </c>
-      <c r="H8" s="18">
-        <v>44252</v>
-      </c>
-      <c r="L8" s="17" t="s">
+      <c r="G12" s="14">
+        <v>31463</v>
+      </c>
+      <c r="H12" s="14">
+        <v>40752</v>
+      </c>
+      <c r="L12" s="13">
+        <v>60172292882</v>
+      </c>
+      <c r="M12" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A13" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" s="14">
+        <v>30494</v>
+      </c>
+      <c r="H13" s="14">
+        <v>40145</v>
+      </c>
+      <c r="L13" s="13">
+        <v>60166945993</v>
+      </c>
+      <c r="M13" s="12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A14" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="M8" s="14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="14" t="s">
+      <c r="G14" s="14">
+        <v>31248</v>
+      </c>
+      <c r="H14" s="14">
+        <v>43140</v>
+      </c>
+      <c r="L14" s="13">
+        <v>60166687720</v>
+      </c>
+      <c r="M14" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A15" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G9" s="18">
-        <v>28742</v>
-      </c>
-      <c r="H9" s="18">
-        <v>44490</v>
-      </c>
-      <c r="L9" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="14" t="s">
+      <c r="C15" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" s="14">
+        <v>26976</v>
+      </c>
+      <c r="H15" s="14">
+        <v>44152</v>
+      </c>
+      <c r="L15" s="13">
+        <v>60123181302</v>
+      </c>
+      <c r="M15" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A16" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="18">
-        <v>24020</v>
-      </c>
-      <c r="H10" s="18">
-        <v>42235</v>
-      </c>
-      <c r="L10" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="M10" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B11" s="14" t="s">
+      <c r="C16" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="14">
+        <v>31555</v>
+      </c>
+      <c r="H16" s="14">
+        <v>43033</v>
+      </c>
+      <c r="L16" s="13">
+        <v>60125679999</v>
+      </c>
+      <c r="M16" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A17" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G11" s="18">
-        <v>31672</v>
-      </c>
-      <c r="H11" s="18">
-        <v>42996</v>
-      </c>
-      <c r="L11" s="17">
-        <v>60127264633</v>
-      </c>
-      <c r="M11" s="14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="14" t="s">
+      <c r="C17" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="14">
+        <v>31638</v>
+      </c>
+      <c r="H17" s="14">
+        <v>43290</v>
+      </c>
+      <c r="L17" s="13">
+        <v>60124155308</v>
+      </c>
+      <c r="M17" s="15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A18" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="18">
-        <v>31359</v>
-      </c>
-      <c r="H12" s="18">
-        <v>41636</v>
-      </c>
-      <c r="L12" s="17">
-        <v>60126617880</v>
-      </c>
-      <c r="M12" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
+      <c r="C18" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="G18" s="14">
+        <v>31657</v>
+      </c>
+      <c r="H18" s="14">
+        <v>42989</v>
+      </c>
+      <c r="L18" s="13">
+        <v>60129203111</v>
+      </c>
+      <c r="M18" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A19" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G13" s="18">
-        <v>31463</v>
-      </c>
-      <c r="H13" s="18">
-        <v>40752</v>
-      </c>
-      <c r="L13" s="17">
-        <v>60172292882</v>
-      </c>
-      <c r="M13" s="14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="14" t="s">
+      <c r="C19" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="14">
+        <v>31834</v>
+      </c>
+      <c r="H19" s="14">
+        <v>42884</v>
+      </c>
+      <c r="L19" s="13">
+        <v>60173197963</v>
+      </c>
+      <c r="M19" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A20" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G14" s="18">
-        <v>30494</v>
-      </c>
-      <c r="H14" s="18">
-        <v>40145</v>
-      </c>
-      <c r="L14" s="17">
-        <v>60166945993</v>
-      </c>
-      <c r="M14" s="14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="16" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="17" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="18" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="19" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="20" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="21" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="22" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="23" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="24" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="25" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="26" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="27" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="28" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="29" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="30" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="31" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="32" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="33" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="34" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="35" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="36" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="37" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="38" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="39" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="40" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="41" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="42" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="43" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="44" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="45" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="46" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="47" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="48" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="49" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="50" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="51" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="52" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="53" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="54" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="55" ht="22" customHeight="1" x14ac:dyDescent="0.35"/>
+      <c r="C20" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="14">
+        <v>31708</v>
+      </c>
+      <c r="H20" s="14">
+        <v>43063</v>
+      </c>
+      <c r="L20" s="13">
+        <v>60193828742</v>
+      </c>
+      <c r="M20" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A21" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="14">
+        <v>25049</v>
+      </c>
+      <c r="H21" s="14">
+        <v>42619</v>
+      </c>
+      <c r="L21" s="13">
+        <v>60123267263</v>
+      </c>
+      <c r="M21" s="15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="22.15" customHeight="1">
+      <c r="A22" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="14">
+        <v>31750</v>
+      </c>
+      <c r="H22" s="14">
+        <v>42976</v>
+      </c>
+      <c r="L22" s="13">
+        <v>60172121039</v>
+      </c>
+      <c r="M22" s="15" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="24" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="25" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="26" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="27" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="28" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="29" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="30" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="31" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="32" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="33" ht="22.15" customHeight="1"/>
+    <row r="34" ht="22.15" customHeight="1"/>
+    <row r="35" ht="22.15" customHeight="1"/>
+    <row r="36" ht="22.15" customHeight="1"/>
+    <row r="37" ht="22.15" customHeight="1"/>
+    <row r="38" ht="22.15" customHeight="1"/>
+    <row r="39" ht="22.15" customHeight="1"/>
+    <row r="40" ht="22.15" customHeight="1"/>
+    <row r="41" ht="22.15" customHeight="1"/>
+    <row r="42" ht="22.15" customHeight="1"/>
+    <row r="43" ht="22.15" customHeight="1"/>
+    <row r="44" ht="22.15" customHeight="1"/>
+    <row r="45" ht="22.15" customHeight="1"/>
+    <row r="46" ht="22.15" customHeight="1"/>
+    <row r="47" ht="22.15" customHeight="1"/>
+    <row r="48" ht="22.15" customHeight="1"/>
+    <row r="49" ht="22.15" customHeight="1"/>
+    <row r="50" ht="22.15" customHeight="1"/>
+    <row r="51" ht="22.15" customHeight="1"/>
+    <row r="52" ht="22.15" customHeight="1"/>
+    <row r="53" ht="22.15" customHeight="1"/>
+    <row r="54" ht="22.15" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B6:B55" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B5:B54" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Active,Prospect,Inactive"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C6:C55" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C5:C54" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Affluent,Mass Affluent,HNW,UHNW"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D6:D55" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D5:D54" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>"Conservative,Moderate,Aggressive"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G6:J55" xr:uid="{00000000-0002-0000-0100-000006000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G5:J54" xr:uid="{00000000-0002-0000-0100-000006000000}">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M14" r:id="rId1" xr:uid="{3D1BFD75-5EC3-494D-9F15-D5D141FA6075}"/>
+    <hyperlink ref="M15" r:id="rId2" xr:uid="{8C1A08C0-9D01-44B4-A145-68B589EC560A}"/>
+    <hyperlink ref="M16" r:id="rId3" xr:uid="{8BA9D6E2-B388-4BA8-924A-4E35A1191A7F}"/>
+    <hyperlink ref="M17" r:id="rId4" xr:uid="{8DB58BB2-8598-43FB-A26C-5DD88CDA6042}"/>
+    <hyperlink ref="M18" r:id="rId5" xr:uid="{8123F5F6-09CC-408C-8255-A1B29AAABE7A}"/>
+    <hyperlink ref="M19" r:id="rId6" xr:uid="{FE4641B7-51B8-4E1B-A0F6-01CB291FA6E5}"/>
+    <hyperlink ref="M20" r:id="rId7" xr:uid="{F44DCFE6-BC4C-4FF2-B4DF-306333993635}"/>
+    <hyperlink ref="M21" r:id="rId8" xr:uid="{C9FD17BF-A78F-4B15-97C7-A3A1EABBABC3}"/>
+    <hyperlink ref="M22" r:id="rId9" xr:uid="{B0591840-7776-4173-A441-9576CE5B330A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: dashboard alert deep-link + auto mark-read + action choices
1. Dashboard 'New Client Correspondence' now links directly to the specific
   email (/emails?thread=) and Email Hub auto-opens that thread.
2. Opening a thread marks it read in Gmail; client-alerts only shows unread,
   so seen correspondence drops off the dashboard automatically.
3. Email detail footer reworked into a clear 'Choose an action' bar:
   AI Draft Reply / Write Reply / Mark Done.

- lib/gmail.ts: markThreadRead()
- thread route marks read on open
- client-alerts route filters to unread only

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/1_Clients_Database.xlsx
+++ b/notion-import-templates/1_Clients_Database.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
   <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D563757-2660-4B04-8139-2E36AF5670CE}"/>
   <bookViews>
@@ -314,7 +314,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -570,6 +570,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -895,14 +899,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C25"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="15" customHeight="1">
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -913,7 +917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="10.15" customHeight="1">
+    <row r="3" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -924,7 +928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="11.1" customHeight="1">
+    <row r="5" spans="1:3" ht="11.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -935,7 +939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="10.15" customHeight="1">
+    <row r="6" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -946,7 +950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="10.15" customHeight="1">
+    <row r="7" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -957,7 +961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="10.15" customHeight="1">
+    <row r="8" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -968,7 +972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="10.15" customHeight="1">
+    <row r="9" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -979,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="10.15" customHeight="1">
+    <row r="10" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -990,7 +994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="10.15" customHeight="1">
+    <row r="11" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1001,7 +1005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="10.15" customHeight="1">
+    <row r="12" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1012,7 +1016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="11.1" customHeight="1">
+    <row r="14" spans="1:3" ht="11.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1023,7 +1027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="10.15" customHeight="1">
+    <row r="15" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1034,7 +1038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="10.15" customHeight="1">
+    <row r="16" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1045,7 +1049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="10.15" customHeight="1">
+    <row r="17" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1056,7 +1060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="10.15" customHeight="1">
+    <row r="18" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1067,7 +1071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="10.15" customHeight="1">
+    <row r="19" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1078,7 +1082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="11.1" customHeight="1">
+    <row r="21" spans="1:3" ht="11.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1089,7 +1093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="10.15" customHeight="1">
+    <row r="22" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1100,7 +1104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="10.15" customHeight="1">
+    <row r="23" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1111,7 +1115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="10.15" customHeight="1">
+    <row r="24" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1122,7 +1126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="10.15" customHeight="1">
+    <row r="25" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1142,7 +1146,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M54"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="36" style="12" customWidth="1"/>
     <col min="2" max="2" width="14" style="12" customWidth="1"/>
@@ -1155,10 +1159,10 @@
     <col min="11" max="11" width="44" style="12" customWidth="1"/>
     <col min="12" max="12" width="20" style="13" customWidth="1"/>
     <col min="13" max="13" width="30" style="12" customWidth="1"/>
-    <col min="14" max="16384" width="8.7109375" style="12"/>
+    <col min="14" max="16384" width="8.73046875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="28.15" customHeight="1">
+    <row r="1" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="16" t="s">
         <v>22</v>
       </c>
@@ -1175,7 +1179,7 @@
       <c r="L1" s="16"/>
       <c r="M1" s="16"/>
     </row>
-    <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1">
+    <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="17" t="s">
         <v>23</v>
       </c>
@@ -1192,7 +1196,7 @@
       <c r="L2" s="17"/>
       <c r="M2" s="17"/>
     </row>
-    <row r="3" spans="1:13" ht="32.1" customHeight="1">
+    <row r="3" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
         <v>24</v>
       </c>
@@ -1233,7 +1237,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="28.15" customHeight="1">
+    <row r="4" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="11" t="s">
         <v>37</v>
       </c>
@@ -1274,7 +1278,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="22.15" customHeight="1">
+    <row r="5" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="12" t="s">
         <v>47</v>
       </c>
@@ -1294,7 +1298,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="22.15" customHeight="1">
+    <row r="6" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="12" t="s">
         <v>51</v>
       </c>
@@ -1314,7 +1318,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="22.15" customHeight="1">
+    <row r="7" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="12" t="s">
         <v>54</v>
       </c>
@@ -1334,7 +1338,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="22.15" customHeight="1">
+    <row r="8" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="12" t="s">
         <v>57</v>
       </c>
@@ -1354,7 +1358,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="22.15" customHeight="1">
+    <row r="9" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="12" t="s">
         <v>60</v>
       </c>
@@ -1374,7 +1378,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="22.15" customHeight="1">
+    <row r="10" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="12" t="s">
         <v>63</v>
       </c>
@@ -1394,7 +1398,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="22.15" customHeight="1">
+    <row r="11" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="12" t="s">
         <v>65</v>
       </c>
@@ -1414,7 +1418,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="22.15" customHeight="1">
+    <row r="12" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="12" t="s">
         <v>67</v>
       </c>
@@ -1434,7 +1438,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="22.15" customHeight="1">
+    <row r="13" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="12" t="s">
         <v>69</v>
       </c>
@@ -1454,7 +1458,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="22.15" customHeight="1">
+    <row r="14" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="12" t="s">
         <v>71</v>
       </c>
@@ -1477,7 +1481,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="22.15" customHeight="1">
+    <row r="15" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="12" t="s">
         <v>74</v>
       </c>
@@ -1500,7 +1504,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="22.15" customHeight="1">
+    <row r="16" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="12" t="s">
         <v>76</v>
       </c>
@@ -1526,7 +1530,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="22.15" customHeight="1">
+    <row r="17" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="12" t="s">
         <v>79</v>
       </c>
@@ -1552,7 +1556,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="22.15" customHeight="1">
+    <row r="18" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="12" t="s">
         <v>81</v>
       </c>
@@ -1578,7 +1582,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="22.15" customHeight="1">
+    <row r="19" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="12" t="s">
         <v>83</v>
       </c>
@@ -1604,7 +1608,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="22.15" customHeight="1">
+    <row r="20" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="12" t="s">
         <v>85</v>
       </c>
@@ -1630,7 +1634,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="22.15" customHeight="1">
+    <row r="21" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="12" t="s">
         <v>87</v>
       </c>
@@ -1656,7 +1660,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="22.15" customHeight="1">
+    <row r="22" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="12" t="s">
         <v>89</v>
       </c>
@@ -1682,38 +1686,38 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="24" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="25" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="26" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="27" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="28" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="29" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="30" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="31" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="32" spans="1:13" ht="22.15" customHeight="1"/>
-    <row r="33" ht="22.15" customHeight="1"/>
-    <row r="34" ht="22.15" customHeight="1"/>
-    <row r="35" ht="22.15" customHeight="1"/>
-    <row r="36" ht="22.15" customHeight="1"/>
-    <row r="37" ht="22.15" customHeight="1"/>
-    <row r="38" ht="22.15" customHeight="1"/>
-    <row r="39" ht="22.15" customHeight="1"/>
-    <row r="40" ht="22.15" customHeight="1"/>
-    <row r="41" ht="22.15" customHeight="1"/>
-    <row r="42" ht="22.15" customHeight="1"/>
-    <row r="43" ht="22.15" customHeight="1"/>
-    <row r="44" ht="22.15" customHeight="1"/>
-    <row r="45" ht="22.15" customHeight="1"/>
-    <row r="46" ht="22.15" customHeight="1"/>
-    <row r="47" ht="22.15" customHeight="1"/>
-    <row r="48" ht="22.15" customHeight="1"/>
-    <row r="49" ht="22.15" customHeight="1"/>
-    <row r="50" ht="22.15" customHeight="1"/>
-    <row r="51" ht="22.15" customHeight="1"/>
-    <row r="52" ht="22.15" customHeight="1"/>
-    <row r="53" ht="22.15" customHeight="1"/>
-    <row r="54" ht="22.15" customHeight="1"/>
+    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="24" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="25" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="26" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="27" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="28" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="29" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="30" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="31" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="32" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="33" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="34" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="35" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="36" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="37" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="38" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="39" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="40" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="41" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="42" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="43" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="44" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="45" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="46" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="47" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="48" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="49" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="50" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="51" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="52" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="53" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="54" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>

</xml_diff>

<commit_message>
feat: Ask ARIA — dashboard daily co-pilot
Adds an ask bar + quick buttons at the top of the dashboard. The assistant
sees a live snapshot of everything actionable (reviews due, follow-ups, new
correspondence, birthdays, expiring policies, recent meetings + action items)
and answers questions like "what's urgent today?" with a ranked, specific
action list using real client names/dates.

- API: POST /api/dashboard-assistant (Gemini with model fallback)
- AskAria component builds context client-side from existing dashboard data

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/1_Clients_Database.xlsx
+++ b/notion-import-templates/1_Clients_Database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D563757-2660-4B04-8139-2E36AF5670CE}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8D8624E-8D6C-4293-92D4-93DBD2FE4978}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="95">
   <si>
     <t/>
   </si>
@@ -308,6 +308,15 @@
   </si>
   <si>
     <t>kayu1204@yahoo.com</t>
+  </si>
+  <si>
+    <t>Mass Affluent</t>
+  </si>
+  <si>
+    <t>JANICE QUEK</t>
+  </si>
+  <si>
+    <t>janiceq1994@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -501,7 +510,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -554,6 +563,9 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -570,10 +582,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1285,6 +1293,12 @@
       <c r="B5" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G5" s="14">
         <v>31769</v>
       </c>
@@ -1305,6 +1319,12 @@
       <c r="B6" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C6" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G6" s="14">
         <v>28299</v>
       </c>
@@ -1325,6 +1345,12 @@
       <c r="B7" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C7" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G7" s="14">
         <v>30150</v>
       </c>
@@ -1345,6 +1371,12 @@
       <c r="B8" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C8" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G8" s="14">
         <v>28742</v>
       </c>
@@ -1365,6 +1397,12 @@
       <c r="B9" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C9" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G9" s="14">
         <v>24020</v>
       </c>
@@ -1385,6 +1423,12 @@
       <c r="B10" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C10" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G10" s="14">
         <v>31672</v>
       </c>
@@ -1405,6 +1449,12 @@
       <c r="B11" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C11" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G11" s="14">
         <v>31359</v>
       </c>
@@ -1425,6 +1475,12 @@
       <c r="B12" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C12" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G12" s="14">
         <v>31463</v>
       </c>
@@ -1445,6 +1501,12 @@
       <c r="B13" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="C13" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G13" s="14">
         <v>30494</v>
       </c>
@@ -1468,6 +1530,9 @@
       <c r="C14" s="12" t="s">
         <v>72</v>
       </c>
+      <c r="D14" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G14" s="14">
         <v>31248</v>
       </c>
@@ -1491,6 +1556,9 @@
       <c r="C15" s="12" t="s">
         <v>72</v>
       </c>
+      <c r="D15" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="G15" s="14">
         <v>26976</v>
       </c>
@@ -1512,7 +1580,7 @@
         <v>48</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>77</v>
@@ -1538,7 +1606,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>77</v>
@@ -1564,7 +1632,7 @@
         <v>48</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>77</v>
@@ -1590,7 +1658,7 @@
         <v>48</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>77</v>
@@ -1616,7 +1684,7 @@
         <v>48</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>77</v>
@@ -1668,15 +1736,15 @@
         <v>48</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="G22" s="14">
+      <c r="G22" s="18">
         <v>31750</v>
       </c>
-      <c r="H22" s="14">
+      <c r="H22" s="18">
         <v>42976</v>
       </c>
       <c r="L22" s="13">
@@ -1686,7 +1754,32 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G23" s="18">
+        <v>34472</v>
+      </c>
+      <c r="H23" s="18">
+        <v>43434</v>
+      </c>
+      <c r="L23" s="13">
+        <v>60176647938</v>
+      </c>
+      <c r="M23" s="13" t="s">
+        <v>94</v>
+      </c>
+    </row>
     <row r="24" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="25" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="26" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
fix: Ask ARIA never drops advisor-created tasks from urgent/agenda answers
Created tasks without a due date were ranked non-urgent and fell outside the
item cap. Now they're always surfaced — appended as 'Also on your list:' if
they don't make the ranked list, and placed under 'Nice to have' in the
morning plan.
</commit_message>
<xml_diff>
--- a/notion-import-templates/1_Clients_Database.xlsx
+++ b/notion-import-templates/1_Clients_Database.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8D8624E-8D6C-4293-92D4-93DBD2FE4978}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="13_ncr:1_{13B59D5D-5EB8-47F8-8AFB-3DB5994BB597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{991CCE82-0F12-4FF3-935D-B8905F7DC969}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -181,6 +181,12 @@
     <t>Active</t>
   </si>
   <si>
+    <t>Affluent</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
     <t>60107607223</t>
   </si>
   <si>
@@ -208,6 +214,9 @@
     <t>KAREN CHEW AI LENG</t>
   </si>
   <si>
+    <t>Mass Affluent</t>
+  </si>
+  <si>
     <t>60123959997</t>
   </si>
   <si>
@@ -250,9 +259,6 @@
     <t>DORIS CHIEW JING TZE</t>
   </si>
   <si>
-    <t>Affluent</t>
-  </si>
-  <si>
     <t>ahtze85@hotmail.com</t>
   </si>
   <si>
@@ -265,9 +271,6 @@
     <t>LIM WOOI KHANG</t>
   </si>
   <si>
-    <t>Moderate</t>
-  </si>
-  <si>
     <t>wk1168@gmail.com</t>
   </si>
   <si>
@@ -310,10 +313,7 @@
     <t>kayu1204@yahoo.com</t>
   </si>
   <si>
-    <t>Mass Affluent</t>
-  </si>
-  <si>
-    <t>JANICE QUEK</t>
+    <t>JANICE QUEK KHANG WEN</t>
   </si>
   <si>
     <t>janiceq1994@gmail.com</t>
@@ -323,7 +323,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -557,14 +557,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -907,14 +907,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" ht="15" customHeight="1">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -925,7 +925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="10.15" customHeight="1">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -936,7 +936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="11.1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" ht="11.1" customHeight="1">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -947,7 +947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" ht="10.15" customHeight="1">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -958,7 +958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" ht="10.15" customHeight="1">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -969,7 +969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" ht="10.15" customHeight="1">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" ht="10.15" customHeight="1">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -991,7 +991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" ht="10.15" customHeight="1">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" ht="10.15" customHeight="1">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" ht="10.15" customHeight="1">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="11.1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" ht="11.1" customHeight="1">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" ht="10.15" customHeight="1">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" ht="10.15" customHeight="1">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" ht="10.15" customHeight="1">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" ht="10.15" customHeight="1">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" ht="10.15" customHeight="1">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1090,7 +1090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="11.1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" ht="11.1" customHeight="1">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" ht="10.15" customHeight="1">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1112,7 +1112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" ht="10.15" customHeight="1">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3" ht="10.15" customHeight="1">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3" ht="10.15" customHeight="1">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1154,7 +1154,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M54"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="36" style="12" customWidth="1"/>
     <col min="2" max="2" width="14" style="12" customWidth="1"/>
@@ -1167,44 +1167,44 @@
     <col min="11" max="11" width="44" style="12" customWidth="1"/>
     <col min="12" max="12" width="20" style="13" customWidth="1"/>
     <col min="13" max="13" width="30" style="12" customWidth="1"/>
-    <col min="14" max="16384" width="8.73046875" style="12"/>
+    <col min="14" max="16384" width="8.7109375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:13" ht="28.15" customHeight="1">
+      <c r="A1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-    </row>
-    <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+    </row>
+    <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1">
+      <c r="A2" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-    </row>
-    <row r="3" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+    </row>
+    <row r="3" spans="1:13" ht="32.1" customHeight="1">
       <c r="A3" s="10" t="s">
         <v>24</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" ht="28.15" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>37</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" ht="22.15" customHeight="1">
       <c r="A5" s="12" t="s">
         <v>47</v>
       </c>
@@ -1294,10 +1294,10 @@
         <v>48</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G5" s="14">
         <v>31769</v>
@@ -1306,24 +1306,24 @@
         <v>42115</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="22.15" customHeight="1">
       <c r="A6" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G6" s="14">
         <v>28299</v>
@@ -1332,24 +1332,24 @@
         <v>44249</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="22.15" customHeight="1">
       <c r="A7" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G7" s="14">
         <v>30150</v>
@@ -1358,24 +1358,24 @@
         <v>44252</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="22.15" customHeight="1">
       <c r="A8" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G8" s="14">
         <v>28742</v>
@@ -1384,24 +1384,24 @@
         <v>44490</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="22.15" customHeight="1">
       <c r="A9" s="12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G9" s="14">
         <v>24020</v>
@@ -1410,24 +1410,24 @@
         <v>42235</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="22.15" customHeight="1">
       <c r="A10" s="12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G10" s="14">
         <v>31672</v>
@@ -1439,21 +1439,21 @@
         <v>60127264633</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="22.15" customHeight="1">
       <c r="A11" s="12" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G11" s="14">
         <v>31359</v>
@@ -1465,21 +1465,21 @@
         <v>60126617880</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="22.15" customHeight="1">
       <c r="A12" s="12" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G12" s="14">
         <v>31463</v>
@@ -1491,21 +1491,21 @@
         <v>60172292882</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="22.15" customHeight="1">
       <c r="A13" s="12" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G13" s="14">
         <v>30494</v>
@@ -1517,21 +1517,21 @@
         <v>60166945993</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="22.15" customHeight="1">
       <c r="A14" s="12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G14" s="14">
         <v>31248</v>
@@ -1543,21 +1543,21 @@
         <v>60166687720</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="22.15" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G15" s="14">
         <v>26976</v>
@@ -1569,21 +1569,21 @@
         <v>60123181302</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="22.15" customHeight="1">
       <c r="A16" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G16" s="14">
         <v>31555</v>
@@ -1595,21 +1595,21 @@
         <v>60125679999</v>
       </c>
       <c r="M16" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="22.15" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G17" s="14">
         <v>31638</v>
@@ -1621,21 +1621,21 @@
         <v>60124155308</v>
       </c>
       <c r="M17" s="15" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="22.15" customHeight="1">
       <c r="A18" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G18" s="14">
         <v>31657</v>
@@ -1647,21 +1647,21 @@
         <v>60129203111</v>
       </c>
       <c r="M18" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="22.15" customHeight="1">
       <c r="A19" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G19" s="14">
         <v>31834</v>
@@ -1673,21 +1673,21 @@
         <v>60173197963</v>
       </c>
       <c r="M19" s="15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="22.15" customHeight="1">
       <c r="A20" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G20" s="14">
         <v>31708</v>
@@ -1699,21 +1699,21 @@
         <v>60193828742</v>
       </c>
       <c r="M20" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="22.15" customHeight="1">
       <c r="A21" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G21" s="14">
         <v>25049</v>
@@ -1725,36 +1725,36 @@
         <v>60123267263</v>
       </c>
       <c r="M21" s="15" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="22.15" customHeight="1">
       <c r="A22" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G22" s="18">
+        <v>91</v>
+      </c>
+      <c r="G22" s="16">
         <v>31750</v>
       </c>
-      <c r="H22" s="18">
+      <c r="H22" s="16">
         <v>42976</v>
       </c>
       <c r="L22" s="13">
         <v>60172121039</v>
       </c>
       <c r="M22" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="22.15" customHeight="1">
       <c r="A23" s="12" t="s">
         <v>93</v>
       </c>
@@ -1762,15 +1762,15 @@
         <v>48</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G23" s="18">
+        <v>91</v>
+      </c>
+      <c r="G23" s="16">
         <v>34472</v>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="16">
         <v>43434</v>
       </c>
       <c r="L23" s="13">
@@ -1780,37 +1780,37 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="25" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="26" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="27" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="28" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="29" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="30" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="31" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="32" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="33" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="34" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="35" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="36" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="37" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="38" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="39" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="40" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="41" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="42" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="43" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="44" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="45" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="46" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="47" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="48" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="49" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="50" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="51" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="52" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="53" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="54" ht="22.15" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="24" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="25" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="26" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="27" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="28" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="29" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="30" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="31" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="32" spans="1:13" ht="22.15" customHeight="1"/>
+    <row r="33" ht="22.15" customHeight="1"/>
+    <row r="34" ht="22.15" customHeight="1"/>
+    <row r="35" ht="22.15" customHeight="1"/>
+    <row r="36" ht="22.15" customHeight="1"/>
+    <row r="37" ht="22.15" customHeight="1"/>
+    <row r="38" ht="22.15" customHeight="1"/>
+    <row r="39" ht="22.15" customHeight="1"/>
+    <row r="40" ht="22.15" customHeight="1"/>
+    <row r="41" ht="22.15" customHeight="1"/>
+    <row r="42" ht="22.15" customHeight="1"/>
+    <row r="43" ht="22.15" customHeight="1"/>
+    <row r="44" ht="22.15" customHeight="1"/>
+    <row r="45" ht="22.15" customHeight="1"/>
+    <row r="46" ht="22.15" customHeight="1"/>
+    <row r="47" ht="22.15" customHeight="1"/>
+    <row r="48" ht="22.15" customHeight="1"/>
+    <row r="49" ht="22.15" customHeight="1"/>
+    <row r="50" ht="22.15" customHeight="1"/>
+    <row r="51" ht="22.15" customHeight="1"/>
+    <row r="52" ht="22.15" customHeight="1"/>
+    <row r="53" ht="22.15" customHeight="1"/>
+    <row r="54" ht="22.15" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>

</xml_diff>